<commit_message>
Update prototype budget breakdown Excel sheet
</commit_message>
<xml_diff>
--- a/Farmanaut_GearX_Hydraulic_Upgrade_Budget_100000-main.xlsx
+++ b/Farmanaut_GearX_Hydraulic_Upgrade_Budget_100000-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karthikkrazy\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5397A68B-4235-418C-8428-D7FFA6D4BE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D70B92-BCCB-4F17-AFF6-FFFF26C3141B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -502,6 +502,7 @@
         <v>22000</v>
       </c>
       <c r="F2">
+        <f>D2*E2</f>
         <v>22000</v>
       </c>
     </row>
@@ -522,6 +523,7 @@
         <v>18000</v>
       </c>
       <c r="F3">
+        <f t="shared" ref="F3:F12" si="0">D3*E3</f>
         <v>18000</v>
       </c>
     </row>
@@ -542,6 +544,7 @@
         <v>8500</v>
       </c>
       <c r="F4">
+        <f t="shared" si="0"/>
         <v>17000</v>
       </c>
     </row>
@@ -562,6 +565,7 @@
         <v>1200</v>
       </c>
       <c r="F5">
+        <f t="shared" si="0"/>
         <v>9600</v>
       </c>
     </row>
@@ -582,6 +586,7 @@
         <v>750</v>
       </c>
       <c r="F6">
+        <f t="shared" si="0"/>
         <v>4500</v>
       </c>
     </row>
@@ -602,6 +607,7 @@
         <v>6500</v>
       </c>
       <c r="F7">
+        <f t="shared" si="0"/>
         <v>6500</v>
       </c>
     </row>
@@ -622,6 +628,7 @@
         <v>2500</v>
       </c>
       <c r="F8">
+        <f t="shared" si="0"/>
         <v>2500</v>
       </c>
     </row>
@@ -642,6 +649,7 @@
         <v>4500</v>
       </c>
       <c r="F9">
+        <f t="shared" si="0"/>
         <v>4500</v>
       </c>
     </row>
@@ -662,6 +670,7 @@
         <v>3200</v>
       </c>
       <c r="F10">
+        <f t="shared" si="0"/>
         <v>3200</v>
       </c>
     </row>
@@ -682,6 +691,7 @@
         <v>5500</v>
       </c>
       <c r="F11">
+        <f t="shared" si="0"/>
         <v>5500</v>
       </c>
     </row>
@@ -699,9 +709,10 @@
         <v>1</v>
       </c>
       <c r="E12">
-        <v>4700</v>
+        <v>6700</v>
       </c>
       <c r="F12">
+        <f t="shared" si="0"/>
         <v>6700</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update prototype budget breakdown Excel sheet once more
</commit_message>
<xml_diff>
--- a/Farmanaut_GearX_Hydraulic_Upgrade_Budget_100000-main.xlsx
+++ b/Farmanaut_GearX_Hydraulic_Upgrade_Budget_100000-main.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karthikkrazy\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karthikkrazy\Downloads\farmonaut-letter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D70B92-BCCB-4F17-AFF6-FFFF26C3141B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4017B41E-8210-44D6-99C4-3C165240AAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,7 +141,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -149,12 +149,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,280 +473,290 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="B1:G15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="32.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="2:7" ht="59.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1">
         <v>22000</v>
       </c>
-      <c r="F2">
-        <f>D2*E2</f>
+      <c r="G3" s="1">
+        <f>E3*F3</f>
         <v>22000</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B4" s="1">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
         <v>18000</v>
       </c>
-      <c r="F3">
-        <f t="shared" ref="F3:F12" si="0">D3*E3</f>
+      <c r="G4" s="1">
+        <f t="shared" ref="G4:G13" si="0">E4*F4</f>
         <v>18000</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5" s="1">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4">
+      <c r="E5" s="1">
         <v>2</v>
       </c>
-      <c r="E4">
+      <c r="F5" s="1">
         <v>8500</v>
       </c>
-      <c r="F4">
+      <c r="G5" s="1">
         <f t="shared" si="0"/>
         <v>17000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B6" s="1">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D5">
+      <c r="E6" s="1">
         <v>8</v>
       </c>
-      <c r="E5">
+      <c r="F6" s="1">
         <v>1200</v>
       </c>
-      <c r="F5">
+      <c r="G6" s="1">
         <f t="shared" si="0"/>
         <v>9600</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B7" s="1">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6">
+      <c r="E7" s="1">
         <v>6</v>
       </c>
-      <c r="E6">
+      <c r="F7" s="1">
         <v>750</v>
       </c>
-      <c r="F6">
+      <c r="G7" s="1">
         <f t="shared" si="0"/>
         <v>4500</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B8" s="1">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1">
         <v>6500</v>
       </c>
-      <c r="F7">
+      <c r="G8" s="1">
         <f t="shared" si="0"/>
         <v>6500</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B9" s="1">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1">
         <v>2500</v>
       </c>
-      <c r="F8">
+      <c r="G9" s="1">
         <f t="shared" si="0"/>
         <v>2500</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10" s="1">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
+      <c r="E10" s="1">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1">
         <v>4500</v>
       </c>
-      <c r="F9">
+      <c r="G10" s="1">
         <f t="shared" si="0"/>
         <v>4500</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B11" s="1">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
+      <c r="E11" s="1">
+        <v>1</v>
+      </c>
+      <c r="F11" s="1">
         <v>3200</v>
       </c>
-      <c r="F10">
+      <c r="G11" s="1">
         <f t="shared" si="0"/>
         <v>3200</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" s="1">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
+      <c r="E12" s="1">
+        <v>1</v>
+      </c>
+      <c r="F12" s="1">
         <v>5500</v>
       </c>
-      <c r="F11">
+      <c r="G12" s="1">
         <f t="shared" si="0"/>
         <v>5500</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B13" s="1">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12">
+      <c r="E13" s="1">
+        <v>1</v>
+      </c>
+      <c r="F13" s="1">
         <v>6700</v>
       </c>
-      <c r="F12">
+      <c r="G13" s="1">
         <f t="shared" si="0"/>
         <v>6700</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="E13" t="s">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F13">
-        <f>SUM(F2:F12)</f>
+      <c r="G14" s="1">
+        <f>SUM(G3:G13)</f>
         <v>100000</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="E14" t="s">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F14">
-        <f>F13</f>
+      <c r="G15" s="1">
+        <f>G14</f>
         <v>100000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update recipient to Registrar Dr. Ravichand Mandalapu, remove From block, update PIN references, and add new attachments section
</commit_message>
<xml_diff>
--- a/Farmanaut_GearX_Hydraulic_Upgrade_Budget_100000-main.xlsx
+++ b/Farmanaut_GearX_Hydraulic_Upgrade_Budget_100000-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karthikkrazy\Downloads\farmonaut-letter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4017B41E-8210-44D6-99C4-3C165240AAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B349D4B9-7A63-4816-B08F-69FD3590748D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -473,290 +473,291 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:G15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="32.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.26953125" customWidth="1"/>
+    <col min="4" max="4" width="3.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="59.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="59.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>22000</v>
+      </c>
+      <c r="F3" s="1">
+        <f>D3*E3</f>
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
+        <v>18000</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" ref="F4:F13" si="0">D4*E4</f>
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1">
+        <v>8500</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1">
+        <v>8</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1200</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="1">
         <v>6</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E7" s="1">
+        <v>750</v>
+      </c>
+      <c r="F7" s="1">
+        <f t="shared" si="0"/>
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <v>6500</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="E3" s="1">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1">
-        <v>22000</v>
-      </c>
-      <c r="G3" s="1">
-        <f>E3*F3</f>
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B4" s="1">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <v>2500</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <v>4500</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="0"/>
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="E4" s="1">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1">
-        <v>18000</v>
-      </c>
-      <c r="G4" s="1">
-        <f t="shared" ref="G4:G13" si="0">E4*F4</f>
-        <v>18000</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B5" s="1">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1">
+        <v>3200</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="0"/>
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="B12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1</v>
+      </c>
+      <c r="E12" s="1">
+        <v>5500</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="0"/>
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="E5" s="1">
-        <v>2</v>
-      </c>
-      <c r="F5" s="1">
-        <v>8500</v>
-      </c>
-      <c r="G5" s="1">
-        <f t="shared" si="0"/>
-        <v>17000</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B6" s="1">
-        <v>4</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="1">
-        <v>8</v>
-      </c>
-      <c r="F6" s="1">
-        <v>1200</v>
-      </c>
-      <c r="G6" s="1">
-        <f t="shared" si="0"/>
-        <v>9600</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B7" s="1">
-        <v>5</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="1">
-        <v>6</v>
-      </c>
-      <c r="F7" s="1">
-        <v>750</v>
-      </c>
-      <c r="G7" s="1">
-        <f t="shared" si="0"/>
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B8" s="1">
-        <v>6</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="1">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1">
-        <v>6500</v>
-      </c>
-      <c r="G8" s="1">
-        <f t="shared" si="0"/>
-        <v>6500</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B9" s="1">
-        <v>7</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1</v>
-      </c>
-      <c r="F9" s="1">
-        <v>2500</v>
-      </c>
-      <c r="G9" s="1">
-        <f t="shared" si="0"/>
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B10" s="1">
-        <v>8</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="1">
-        <v>1</v>
-      </c>
-      <c r="F10" s="1">
-        <v>4500</v>
-      </c>
-      <c r="G10" s="1">
-        <f t="shared" si="0"/>
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B11" s="1">
-        <v>9</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="1">
-        <v>1</v>
-      </c>
-      <c r="F11" s="1">
-        <v>3200</v>
-      </c>
-      <c r="G11" s="1">
-        <f t="shared" si="0"/>
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="1">
-        <v>10</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="1">
-        <v>1</v>
-      </c>
-      <c r="F12" s="1">
-        <v>5500</v>
-      </c>
-      <c r="G12" s="1">
-        <f t="shared" si="0"/>
-        <v>5500</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B13" s="1">
-        <v>11</v>
+      <c r="B13" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
       <c r="E13" s="1">
-        <v>1</v>
+        <v>6700</v>
       </c>
       <c r="F13" s="1">
+        <f t="shared" si="0"/>
         <v>6700</v>
       </c>
-      <c r="G13" s="1">
-        <f t="shared" si="0"/>
-        <v>6700</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="1">
-        <f>SUM(G3:G13)</f>
+      <c r="F14" s="1">
+        <f>SUM(F3:F13)</f>
         <v>100000</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="1">
-        <f>G14</f>
+      <c r="F15" s="1">
+        <f>F14</f>
         <v>100000</v>
       </c>
     </row>

</xml_diff>